<commit_message>
Update README.md with project setup instructions and usage details
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mandini\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9EDDAB-3B82-410C-9D7F-A70C4A5F598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8608379-8882-40FC-A87B-B4999CD81ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="209">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -40,36 +40,36 @@
     <t>Status</t>
   </si>
   <si>
+    <t>eeka litr keeyda?</t>
+  </si>
+  <si>
+    <t>ඒක ලීටර් කීයද?</t>
+  </si>
+  <si>
+    <t>ada hire keeyk giyda?</t>
+  </si>
+  <si>
+    <t>අද හයර් කීයක් ගියාද?</t>
+  </si>
+  <si>
+    <t>wahaama eka eyata denna.</t>
+  </si>
+  <si>
+    <t>වහාම ඒක එයාට දෙන්න.</t>
+  </si>
+  <si>
     <t>Neg_0001</t>
   </si>
   <si>
+    <t>Neg_0002</t>
+  </si>
+  <si>
+    <t>Neg_0003</t>
+  </si>
+  <si>
     <t>s</t>
   </si>
   <si>
-    <t>eeka litr keeyda?</t>
-  </si>
-  <si>
-    <t>ඒක ලීටර් කීයද?</t>
-  </si>
-  <si>
-    <t>Neg_0002</t>
-  </si>
-  <si>
-    <t>ada hire keeyk giyda?</t>
-  </si>
-  <si>
-    <t>අද හයර් කීයක් ගියාද?</t>
-  </si>
-  <si>
-    <t>Neg_0003</t>
-  </si>
-  <si>
-    <t>wahaama eka eyata denna.</t>
-  </si>
-  <si>
-    <t>වහාම ඒක එයාට දෙන්න.</t>
-  </si>
-  <si>
     <t>Neg_0004</t>
   </si>
   <si>
@@ -82,99 +82,99 @@
     <t>Neg_0005</t>
   </si>
   <si>
+    <t>suba udasanak, apge shakawata obawa sadarayen piliganimu.</t>
+  </si>
+  <si>
+    <t>සුබ උදෑසනක්, අපගේ ශාඛාවට ඔබව සාදරයෙන් පිළිගනිමු</t>
+  </si>
+  <si>
+    <t>Neg_0006</t>
+  </si>
+  <si>
+    <t>oyage usas vimata ape suba pathum.</t>
+  </si>
+  <si>
+    <t>ඔයාගේ උසස් වීමට අපේ සුබ පැතුම්.</t>
+  </si>
+  <si>
+    <t>Neg_0007</t>
+  </si>
+  <si>
+    <t>eyta kiyanna puluwannam mge paana genna kiyla.</t>
+  </si>
+  <si>
+    <t>එයාට කියන්න පුලුවන්නම් මගේ පෑන ගේන්න කියලා.</t>
+  </si>
+  <si>
+    <t>Neg_0008</t>
+  </si>
+  <si>
+    <t>ane a kaden kema ekak gennako.</t>
+  </si>
+  <si>
+    <t>අනේ ඒ කඩෙන් කෑම එකක් ගේන්නකෝ.</t>
+  </si>
+  <si>
+    <t>Neg_0009</t>
+  </si>
+  <si>
+    <t>hari, mn eka gennm.</t>
+  </si>
+  <si>
+    <t>හරි, මන් ඒක ගේන්නම්.</t>
+  </si>
+  <si>
+    <t>Neg_0010</t>
+  </si>
+  <si>
+    <t>eka litr 10i.</t>
+  </si>
+  <si>
+    <t>ඒක ලීටර් 10යි.</t>
+  </si>
+  <si>
+    <t>Neg_0011</t>
+  </si>
+  <si>
+    <t>pata pata pansal godai.</t>
+  </si>
+  <si>
+    <t>පාට පාට පැන්සල් ගොඩයි.</t>
+  </si>
+  <si>
+    <t>Neg_0012</t>
+  </si>
+  <si>
+    <t>hu hu kiygena kochchiyk enwa anna.</t>
+  </si>
+  <si>
+    <t>හූ හූ කියාගෙන කෝච්චියක් එනවා අන්න.</t>
+  </si>
+  <si>
+    <t>Neg_0013</t>
+  </si>
+  <si>
+    <t>Neg_0014</t>
+  </si>
+  <si>
+    <t>"hari, mn krannm" akka kiwwa.</t>
+  </si>
+  <si>
+    <t>"හරි, මන් කරන්නම්" අක්කා කිව්වා.</t>
+  </si>
+  <si>
+    <t>Neg_0015</t>
+  </si>
+  <si>
+    <t>"siyalla naesena suluiy, nopamawa kusal wadanna." pothaka thibbe.</t>
+  </si>
+  <si>
     <t>m</t>
   </si>
   <si>
-    <t>suba udasanak, apge shakawata obawa sadarayen piliganimu.</t>
-  </si>
-  <si>
-    <t>සුබ උදෑසනක්, අපගේ ශාඛාවට ඔබව සාදරයෙන් පිළිගනිමු</t>
-  </si>
-  <si>
-    <t>Neg_0006</t>
-  </si>
-  <si>
-    <t>oyage usas vimata ape suba pathum.</t>
-  </si>
-  <si>
-    <t>ඔයාගේ උසස් වීමට අපේ සුබ පැතුම්.</t>
-  </si>
-  <si>
-    <t>Neg_0007</t>
-  </si>
-  <si>
-    <t>eyta kiyanna puluwannam mge paana genna kiyla.</t>
-  </si>
-  <si>
-    <t>එයාට කියන්න පුලුවන්නම් මගේ පෑන ගේන්න කියලා.</t>
-  </si>
-  <si>
-    <t>Neg_0008</t>
-  </si>
-  <si>
-    <t>ane a kaden kema ekak gennako.</t>
-  </si>
-  <si>
-    <t>අනේ ඒ කඩෙන් කෑම එකක් ගේන්නකෝ.</t>
-  </si>
-  <si>
-    <t>Neg_0009</t>
-  </si>
-  <si>
-    <t>hari, mn eka gennm.</t>
-  </si>
-  <si>
-    <t>හරි, මන් ඒක ගේන්නම්.</t>
-  </si>
-  <si>
-    <t>Neg_0010</t>
-  </si>
-  <si>
-    <t>eka litr 10i.</t>
-  </si>
-  <si>
-    <t>ඒක ලීටර් 10යි.</t>
-  </si>
-  <si>
-    <t>Neg_0011</t>
-  </si>
-  <si>
-    <t>pata pata pansal godai.</t>
-  </si>
-  <si>
-    <t>පාට පාට පැන්සල් ගොඩයි.</t>
-  </si>
-  <si>
-    <t>Neg_0012</t>
-  </si>
-  <si>
-    <t>hu hu kiygena kochchiyk enwa anna.</t>
-  </si>
-  <si>
-    <t>හූ හූ කියාගෙන කෝච්චියක් එනවා අන්න.</t>
-  </si>
-  <si>
-    <t>Neg_0013</t>
-  </si>
-  <si>
-    <t>"hari, mn krannm" akka kiwwa.</t>
-  </si>
-  <si>
-    <t>"හරි, මන් කරන්නම්" අක්කා කිව්වා.</t>
-  </si>
-  <si>
-    <t>Neg_0014</t>
-  </si>
-  <si>
-    <t>"siyalla naesena suluiy, nopamawa kusal wadanna." pothaka thibbe.</t>
-  </si>
-  <si>
     <t>"සියල්ල නැසෙන සුළුයි, නොපමාව කුසල් වඩන්න."පොතක තිබ්බේ.</t>
   </si>
   <si>
-    <t>Neg_0015</t>
-  </si>
-  <si>
     <t>mm eyta withrai adare.</t>
   </si>
   <si>
@@ -229,278 +229,431 @@
     <t>Neg_0021</t>
   </si>
   <si>
+    <t>oyge vm eke dns wdada?</t>
+  </si>
+  <si>
+    <t>ඔයාගේ vm එකේ dns වැඩද?</t>
+  </si>
+  <si>
+    <t>Neg_0022</t>
+  </si>
+  <si>
+    <t>oya smtp gna dnnwda?</t>
+  </si>
+  <si>
+    <t>ඔයා smtp ගැන දන්නවාද?</t>
+  </si>
+  <si>
+    <t>Neg_0023</t>
+  </si>
+  <si>
+    <t>mn eka eduscope eken gththe.</t>
+  </si>
+  <si>
+    <t>මන් ඒක eduscope එකෙන් ගත්තේ.</t>
+  </si>
+  <si>
+    <t>Neg_0024</t>
+  </si>
+  <si>
+    <t>mn eka temu eken order kla.</t>
+  </si>
+  <si>
+    <t>මන් ඒක temu එකෙන් order කළා.</t>
+  </si>
+  <si>
+    <t>Neg_0025</t>
+  </si>
+  <si>
+    <t>Neg_0026</t>
+  </si>
+  <si>
+    <t>Neg_0027</t>
+  </si>
+  <si>
+    <t>mn heta pitch krnwa.</t>
+  </si>
+  <si>
+    <t>මන් හෙට pitch කරනවා.</t>
+  </si>
+  <si>
+    <t>Neg_0028</t>
+  </si>
+  <si>
+    <t>mta heta race ekak thiyenwa.</t>
+  </si>
+  <si>
+    <t>මට හෙට race එකක් තියෙනවා.</t>
+  </si>
+  <si>
+    <t>Neg_0029</t>
+  </si>
+  <si>
+    <t>api ada raa switzerland ynwa.</t>
+  </si>
+  <si>
+    <t>අපි අද රෑ switzerland යනවා.</t>
+  </si>
+  <si>
+    <t>Neg_0030</t>
+  </si>
+  <si>
+    <t>mn vietnam gihin thiyenwa.</t>
+  </si>
+  <si>
+    <t>මන් vietnam ගිහින් තියෙනවා.</t>
+  </si>
+  <si>
+    <t>Neg_0031</t>
+  </si>
+  <si>
+    <t>kohli top level batsman kenek.</t>
+  </si>
+  <si>
+    <t>කෝලි ටොප් ලෙවල් බට්ස්මන් කෙනෙක්.</t>
+  </si>
+  <si>
+    <t>Neg_0032</t>
+  </si>
+  <si>
+    <t>sachithra ada rata ynwa.</t>
+  </si>
+  <si>
+    <t>සචිත්‍ර අද රට යනවා.</t>
+  </si>
+  <si>
+    <t>Neg_0033</t>
+  </si>
+  <si>
+    <t>Neg_0034</t>
+  </si>
+  <si>
+    <t>api hotel eke dws 6k idiya. ekn 3kma awidinna giya.</t>
+  </si>
+  <si>
+    <t>අපි හොටෙල් එකේ දවස් 6ක් ගියා. ඒකෙන් 3ක්ම ඇවිදින්න ගියා.</t>
+  </si>
+  <si>
+    <t>mge processor eka 4th gen ekak.</t>
+  </si>
+  <si>
+    <t>මගේ ප්රොසෙසර් එක 4th ජෙන් එකක්.</t>
+  </si>
+  <si>
+    <t>Neg_0035</t>
+  </si>
+  <si>
+    <t>mata japan yen 100k hambuna.</t>
+  </si>
+  <si>
+    <t>මට ජපන් යෙන් 100ක් හම්බුණා.</t>
+  </si>
+  <si>
+    <t>Neg_0036</t>
+  </si>
+  <si>
+    <t>Neg_0037</t>
+  </si>
+  <si>
+    <t>ada session eka 9.30 a.m. wlata thiyenne.</t>
+  </si>
+  <si>
+    <t>අද session එක 9.30 a.m. වලට තියෙන්නේ.</t>
+  </si>
+  <si>
+    <t>Neg_0038</t>
+  </si>
+  <si>
+    <t>ape mama dan sahena kalayak wada krna nisa riyal 2000k padi labenwa.</t>
+  </si>
+  <si>
+    <t>heta class eke bell eka 10.00a.m. wlata ghnna kiyla sir kiwwa.</t>
+  </si>
+  <si>
+    <t>හෙට class එකේ bell එක 10.00a.m. වලට ගහන්න කියලා sir කිව්වා.</t>
+  </si>
+  <si>
+    <t>Neg_0039</t>
+  </si>
+  <si>
+    <t>interview eka thiyenwa kiyla amma kiwwe june 7.</t>
+  </si>
+  <si>
+    <t>interview එක තියෙනවා කියලා අම්මා කිව්වේ june 7.</t>
+  </si>
+  <si>
+    <t>Neg_0040</t>
+  </si>
+  <si>
+    <t>api a gamana ynna dagamau ammala ekka may 30 wge.</t>
+  </si>
+  <si>
+    <t>අපි ආ ගමන යන්න දාගමූ අම්මලා එක්ක may 30 වගේ.</t>
+  </si>
+  <si>
+    <t>Neg_0041</t>
+  </si>
+  <si>
+    <t>mn hithnne a wathura tankiya litr 1000k.</t>
+  </si>
+  <si>
+    <t>මන් හිතන්නේ ඒ වතුර ටැංකිය ලීට්ර් 1000ක්.</t>
+  </si>
+  <si>
+    <t>Neg_0042</t>
+  </si>
+  <si>
+    <t>Neg_0043</t>
+  </si>
+  <si>
+    <t>ape game idn eheta thiyenwa kilomitr 130k.</t>
+  </si>
+  <si>
+    <t>අපේ ගමේ ඉඳන් එහෙට තියෙනවා කිලෝමීටර් 130ක්.</t>
+  </si>
+  <si>
+    <t>Neg_0044</t>
+  </si>
+  <si>
+    <t>adee mchn elakirine, eka maruwta thiyenwa suddah.</t>
+  </si>
+  <si>
+    <t>අඩේ මචන් එළකිරිනේ, ඒක මරුවට තියෙනවා සුද්දහ්.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">me bajar eke a wge dial ekak na bn. </t>
+  </si>
+  <si>
+    <t>මේ බජාර් එකේ ඒ වගේ ඩයල් එකක් නෑ බන්.</t>
+  </si>
+  <si>
+    <t>Neg_0045</t>
+  </si>
+  <si>
+    <t>poddk me website eka blnna : https://www.slithm.edu.lk/</t>
+  </si>
+  <si>
+    <t>පොඩ්ඩක් මේ website එක බලන්න : https://www.slithm.edu.lk/</t>
+  </si>
+  <si>
+    <t>Neg_0046</t>
+  </si>
+  <si>
+    <t>me mail address ekata ywnna mail eka : edu123@gmail.com</t>
+  </si>
+  <si>
+    <t>මේ mail address එකට යවන්න mail එක : edu123@gmail.com</t>
+  </si>
+  <si>
+    <t>Neg_0047</t>
+  </si>
+  <si>
+    <t>Neg_0048</t>
+  </si>
+  <si>
+    <t>mn ammata hari adarei 🥰.</t>
+  </si>
+  <si>
+    <t>මන් අම්මට හරි ආදරෙයි 🥰.</t>
+  </si>
+  <si>
+    <t>Neg_0049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adanm mta hari tharahai 😡. </t>
+  </si>
+  <si>
+    <t>අදනම් මට හරි තරහයි 😡.</t>
+  </si>
+  <si>
+    <t>a paththen ynna tikk amru wei habai.</t>
+  </si>
+  <si>
+    <t>ඒ පැත්තෙන් යන්න ටිකක් අමාරු වෙයි හැබැයි.</t>
+  </si>
+  <si>
+    <t>Neg_0050</t>
+  </si>
+  <si>
+    <t>api yna gaman eylat eka aran a paren ymu.</t>
+  </si>
+  <si>
+    <t>අපි යන ගමන් එයාලාට ඒක අරන් ඒ පාරෙන් යමු.</t>
+  </si>
+  <si>
     <t>log wenna blnna poddk.</t>
   </si>
   <si>
     <t>log වෙන්න බලන්න පොඩ්ඩක්.</t>
   </si>
   <si>
-    <t>Neg_0022</t>
+    <t>git එකේ pull එකක් ගන්න බලලා.</t>
   </si>
   <si>
     <t>git eke pull ekak gnna balala.</t>
   </si>
   <si>
-    <t>git එකේ pull එකක් ගන්න බලලා.</t>
-  </si>
-  <si>
-    <t>Neg_0023</t>
-  </si>
-  <si>
-    <t>mn eka eduscope eken gththe.</t>
-  </si>
-  <si>
-    <t>මන් ඒක eduscope එකෙන් ගත්තේ.</t>
-  </si>
-  <si>
-    <t>Neg_0024</t>
-  </si>
-  <si>
-    <t>mn eka temu eken order kla.</t>
-  </si>
-  <si>
-    <t>මන් ඒක temu එකෙන් order කළා.</t>
-  </si>
-  <si>
-    <t>Neg_0025</t>
-  </si>
-  <si>
-    <t>oyge vm eke dns wdada?</t>
-  </si>
-  <si>
-    <t>ඔයාගේ vm එකේ dns වැඩද?</t>
-  </si>
-  <si>
-    <t>Neg_0026</t>
-  </si>
-  <si>
-    <t>oya smtp gna dnnwda?</t>
-  </si>
-  <si>
-    <t>ඔයා smtp ගැන දන්නවාද?</t>
-  </si>
-  <si>
-    <t>Neg_0027</t>
-  </si>
-  <si>
-    <t>mn heta pitch krnwa.</t>
-  </si>
-  <si>
-    <t>මන් හෙට pitch කරනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0028</t>
-  </si>
-  <si>
-    <t>mta heta race ekak thiyenwa.</t>
-  </si>
-  <si>
-    <t>මට හෙට race එකක් තියෙනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0029</t>
-  </si>
-  <si>
-    <t>api ada raa switzerland ynwa.</t>
-  </si>
-  <si>
-    <t>අපි අද රෑ switzerland යනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0030</t>
-  </si>
-  <si>
-    <t>mn vietnam gihin thiyenwa.</t>
-  </si>
-  <si>
-    <t>මන් vietnam ගිහින් තියෙනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0031</t>
-  </si>
-  <si>
-    <t>kohli top level batsman kenek.</t>
-  </si>
-  <si>
-    <t>කෝලි ටොප් ලෙවල් බට්ස්මන් කෙනෙක්.</t>
-  </si>
-  <si>
-    <t>Neg_0032</t>
-  </si>
-  <si>
-    <t>sachithra ada rata ynwa.</t>
-  </si>
-  <si>
-    <t>සචිත්‍ර අද රට යනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0033</t>
-  </si>
-  <si>
-    <t>mge processor eka 4th gen ekak.</t>
-  </si>
-  <si>
-    <t>මගේ ප්රොසෙසර් එක 4th ජෙන් එකක්.</t>
-  </si>
-  <si>
-    <t>Neg_0034</t>
-  </si>
-  <si>
-    <t>api hotel eke dws 6k idiya. ekn 3kma awidinna giya.</t>
-  </si>
-  <si>
-    <t>අපි හොටෙල් එකේ දවස් 6ක් ගියා. ඒකෙන් 3ක්ම ඇවිදින්න ගියා.</t>
-  </si>
-  <si>
-    <t>Neg_0035</t>
-  </si>
-  <si>
-    <t>mata japan yen 100k hambuna.</t>
-  </si>
-  <si>
-    <t>මට ජපන් යෙන් 100ක් හම්බුණා.</t>
-  </si>
-  <si>
-    <t>Neg_0036</t>
-  </si>
-  <si>
-    <t>ape mama dan sahena kalayak wada krna nisa riyal 2000k padi labenwa.</t>
-  </si>
-  <si>
-    <t>අපේ මාමා දැන් සෑහෙන කාලයක් වැඩ කරන නිසා riyal 2000ක් පඩි ලබෙනවා.</t>
-  </si>
-  <si>
-    <t>Neg_0037</t>
-  </si>
-  <si>
-    <t>ada session eka 9.30 a.m. wlata thiyenne.</t>
-  </si>
-  <si>
-    <t>අද session එක 9.30 a.m. වලට තියෙන්නේ.</t>
-  </si>
-  <si>
-    <t>Neg_0038</t>
-  </si>
-  <si>
-    <t>heta class eke bell eka 10.00a.m. wlata ghnna kiyla sir kiwwa.</t>
-  </si>
-  <si>
-    <t>හෙට class එකේ bell එක 10.00a.m. වලට ගහන්න කියලා sir කිව්වා.</t>
-  </si>
-  <si>
-    <t>Neg_0039</t>
-  </si>
-  <si>
-    <t>interview eka thiyenwa kiyla amma kiwwe june 7.</t>
-  </si>
-  <si>
-    <t>interview එක තියෙනවා කියලා අම්මා කිව්වේ june 7.</t>
-  </si>
-  <si>
-    <t>Neg_0040</t>
-  </si>
-  <si>
-    <t>api a gamana ynna dagamau ammala ekka may 30 wge.</t>
-  </si>
-  <si>
-    <t>අපි ආ ගමන යන්න දාගමූ අම්මලා එක්ක may 30 වගේ.</t>
-  </si>
-  <si>
-    <t>Neg_0041</t>
-  </si>
-  <si>
-    <t>mn hithnne a wathura tankiya litr 1000k.</t>
-  </si>
-  <si>
-    <t>මන් හිතන්නේ ඒ වතුර ටැංකිය ලීට්ර් 1000ක්.</t>
-  </si>
-  <si>
-    <t>Neg_0042</t>
-  </si>
-  <si>
-    <t>ape game idn eheta thiyenwa kilomitr 130k.</t>
-  </si>
-  <si>
-    <t>අපේ ගමේ ඉඳන් එහෙට තියෙනවා කිලෝමීටර් 130ක්.</t>
-  </si>
-  <si>
-    <t>Neg_0043</t>
-  </si>
-  <si>
-    <t>adee mchn elakirine, eka maruwta thiyenwa suddah.</t>
-  </si>
-  <si>
-    <t>අඩේ මචන් එළකිරිනේ, ඒක මරුවට තියෙනවා සුද්දහ්.</t>
-  </si>
-  <si>
-    <t>Neg_0044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">me bajar eke a wge dial ekak na bn. </t>
-  </si>
-  <si>
-    <t>මේ බජාර් එකේ ඒ වගේ ඩයල් එකක් නෑ බන්.</t>
-  </si>
-  <si>
-    <t>Neg_0045</t>
-  </si>
-  <si>
-    <t>poddk me website eka blnna : https://www.slithm.edu.lk/</t>
-  </si>
-  <si>
-    <t>පොඩ්ඩක් මේ website එක බලන්න : https://www.slithm.edu.lk/</t>
-  </si>
-  <si>
-    <t>Neg_0046</t>
-  </si>
-  <si>
-    <t>me mail address ekata ywnna mail eka : edu123@gmail.com</t>
-  </si>
-  <si>
-    <t>මේ mail address එකට යවන්න mail එක : edu123@gmail.com</t>
-  </si>
-  <si>
-    <t>Neg_0047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adanm mta hari tharahai 😡. </t>
-  </si>
-  <si>
-    <t>අදනම් මට හරි තරහයි 😡.</t>
-  </si>
-  <si>
-    <t>Neg_0048</t>
-  </si>
-  <si>
-    <t>mn ammata hari adarei 🥰.</t>
-  </si>
-  <si>
-    <t>මන් අම්මට හරි ආදරෙයි 🥰.</t>
-  </si>
-  <si>
-    <t>Neg_0049</t>
-  </si>
-  <si>
-    <t>a paththen ynna tikk amru wei habai.</t>
-  </si>
-  <si>
-    <t>ඒ පැත්තෙන් යන්න ටිකක් අමාරු වෙයි හැබැයි.</t>
-  </si>
-  <si>
-    <t>Neg_0050</t>
-  </si>
-  <si>
-    <t>api yna gaman eylat eka aran a paren ymu.</t>
-  </si>
-  <si>
-    <t>අපි යන ගමන් එයාලාට ඒක අරන් ඒ පාරෙන් යමු.</t>
+    <t>ඒක ලිට්ර් කීය්ද?</t>
+  </si>
+  <si>
+    <t>අද හිරේ කීයක් ගියාද?</t>
+  </si>
+  <si>
+    <t>වහාම එක එයාට දෙන්න.</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>කරුණාකරලා, මගේ පණ මට දෙන්න.</t>
+  </si>
+  <si>
+    <t>සුබ උදසනක්, අපගේ ශාඛාවට ඔබව සාදරයෙන් පිළිගනිමු.</t>
+  </si>
+  <si>
+    <t>ඔයාගෙ උසස් විමට අපේ සුබ පතුම්.</t>
+  </si>
+  <si>
+    <t>එයාට කියන්න පුලුවන්නම් මගේ පාන ගේන්න කියලා.</t>
+  </si>
+  <si>
+    <t>අනේ ආ කඩෙන් කෑම එකක් ගෙන්නකෝ.</t>
+  </si>
+  <si>
+    <t>හරි, මන් ඒක ගෙන්නම්.</t>
+  </si>
+  <si>
+    <t>ඒක ලිටර් 10යි.</t>
+  </si>
+  <si>
+    <t>හු හු කියාගෙන කෝච්චියක් එනවා අන්න.</t>
+  </si>
+  <si>
+    <t>හරි, මන් කරන්නම් අක්කා කිව්වා.</t>
+  </si>
+  <si>
+    <t>ම්ම් එයාට විතරයි ආදරේ.</t>
+  </si>
+  <si>
+    <t>පාට පාට පන්සල් ගොඩයි.</t>
+  </si>
+  <si>
+    <t>මන් හයියෙන් කාගහුවා කියලා එයා මට කාගහනවා.</t>
+  </si>
+  <si>
+    <t>අපි වැඩ කරන ගමන්.</t>
+  </si>
+  <si>
+    <t>මන්‍යෝඝුර්ට් ගෙනාවා.</t>
+  </si>
+  <si>
+    <t>මන් අද campus ගියේ bike එකේ නිසා වැස්සට තෙමුණා නිසා දැන් මට feeling very cold.</t>
+  </si>
+  <si>
+    <t>මන් office එකේ අද leave එක නිසා මට official වැඩ වලට call ගන්න එපා.</t>
+  </si>
+  <si>
+    <t>ලොග් වෙන්න බලන්න පොඩ්ඩක්.</t>
+  </si>
+  <si>
+    <t>ගිට් එකේ පුල් එකක් ගන්න බලලා.</t>
+  </si>
+  <si>
+    <t>මන් ඒක ඇඩුස්කෝපේ එකෙන් ගත්තේ.</t>
+  </si>
+  <si>
+    <t>මන් ඒක ටේමේ එකෙන් order කළා.</t>
+  </si>
+  <si>
+    <t>ඔයා ස්මාට්පී ගැන දන්නවාද?</t>
+  </si>
+  <si>
+    <t>ඔයාගේ වම් එකේ දෑන්ස් වැඩද?</t>
+  </si>
+  <si>
+    <t>මන් හෙට පිට්ච් කරනවා.</t>
+  </si>
+  <si>
+    <t>මට හෙට රෑස් එකක් තියෙනවා.</t>
+  </si>
+  <si>
+    <t>මන් විටම ගිහින් තියෙනවා.</t>
+  </si>
+  <si>
+    <t>අපි අද රෑ ස්විට්සෙර්ලන්ඩ් යනවා.</t>
+  </si>
+  <si>
+    <t>කොහ්ලි ටොප් ලෙෆ් බට්ස්මන් කෙනෙක්.</t>
+  </si>
+  <si>
+    <t>සචිත්ර අද රට යනවා.</t>
+  </si>
+  <si>
+    <t>මගේ ප්රොසෙසර් එක 4ත් ගෙන් එකක්.</t>
+  </si>
+  <si>
+    <t>මට ජපන්‍යෙන් 100ක් හම්බුණා.</t>
+  </si>
+  <si>
+    <t>අපි හොටෙල් එකේ දවස් 6ක් ගියා. එකෙන් 3ක්ම ඇවිදින්න ගියා.</t>
+  </si>
+  <si>
+    <t>අපේ මාමා දැන් සෑහෙන කාලයක් වැඩ කරන නිසා riyal 2000ක් පඩි ලැබෙනවා.</t>
+  </si>
+  <si>
+    <t>අපේ මම දැන් සෑහෙන කාලයක් වැඩ කරන නිසා රියල් 2000ක් පඩි ලබෙනවා.</t>
+  </si>
+  <si>
+    <t>අද session එක 9.30 ආ.ම්. වලට තියෙන්නේ.</t>
+  </si>
+  <si>
+    <t>අපි යන ගමන් එයාලාට් එක අරන් ආ පාරෙන් යමු.</t>
+  </si>
+  <si>
+    <t>ආ පැත්තෙන් යන්න ටිකක් අමාරු වෙයි හැබැයි.</t>
+  </si>
+  <si>
+    <t>මන් අම්මට හරි ආදරෙයි.</t>
+  </si>
+  <si>
+    <t>අදනම් මට හරි තරහයි 🤣.</t>
+  </si>
+  <si>
+    <t>මේ mail address එකට යවන්න mail එක : එදූ123@gmail.කොම්</t>
+  </si>
+  <si>
+    <t>මේ බජර් එකේ ආ වගේ dial එකක් නෑ බන්.</t>
+  </si>
+  <si>
+    <t>"සියල්ල නැසෙන සුළුයි, නොපමාව කුසල් වඩන්න.පොතක තිබ්බේ.</t>
+  </si>
+  <si>
+    <t>අපේ ගමේ ඉඳන් එහෙට තියෙනවා කිලෝමිටර් 130ක්.</t>
+  </si>
+  <si>
+    <t>අඩේ මචන් එළකිරිනේ, ඒක මාරුවට තියෙනවා සුද්දහ්.</t>
+  </si>
+  <si>
+    <t>හෙට class එකේ bell එක 10.00a.ම්. වලට ගහන්න කියලා sir කිව්වා.</t>
+  </si>
+  <si>
+    <t>interview එක තියෙනවා කියලා අම්මා කිව්වේ ජූනේ 7.</t>
+  </si>
+  <si>
+    <t>මන් හිතන්නේ ආ වතුර ටැංකිය ලිටර් 1000ක්.</t>
+  </si>
+  <si>
+    <t>අපි ආ ගමන යන්න දාගමූ අම්මලා එක්ක මැයි 30 වගේ.</t>
+  </si>
+  <si>
+    <t>පොඩ්ඩක් මේ website එක බලන්න : https://www.ස්ලිත්ම්.ඇඩු.ල්ක්/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -532,6 +685,12 @@
       <color theme="1"/>
       <name val="Iskoola Pota"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -599,21 +758,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -928,20 +1087,24 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="5"/>
+      <c r="E2" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
@@ -968,20 +1131,24 @@
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="5"/>
+      <c r="A6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
@@ -1008,20 +1175,24 @@
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="5"/>
+      <c r="C10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
@@ -1048,20 +1219,24 @@
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="5"/>
+      <c r="E14" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="15" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -1088,20 +1263,24 @@
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="5"/>
+      <c r="E18" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
@@ -1128,20 +1307,24 @@
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="5"/>
+      <c r="E22" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
@@ -1168,20 +1351,24 @@
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="5"/>
+      <c r="E26" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
@@ -1208,20 +1395,24 @@
       <c r="F29" s="4"/>
     </row>
     <row r="30" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E30" s="6"/>
-      <c r="F30" s="5"/>
+      <c r="E30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
@@ -1248,20 +1439,24 @@
       <c r="F33" s="4"/>
     </row>
     <row r="34" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D34" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34" s="6"/>
-      <c r="F34" s="5"/>
+      <c r="E34" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
@@ -1288,20 +1483,24 @@
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D38" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E38" s="6"/>
-      <c r="F38" s="5"/>
+      <c r="E38" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="39" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
@@ -1328,20 +1527,24 @@
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D42" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E42" s="6"/>
-      <c r="F42" s="5"/>
+      <c r="E42" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="43" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
@@ -1368,20 +1571,24 @@
       <c r="F45" s="4"/>
     </row>
     <row r="46" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7" t="s">
+      <c r="A46" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B46" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D46" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E46" s="6"/>
-      <c r="F46" s="5"/>
+      <c r="E46" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="47" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
@@ -1408,20 +1615,24 @@
       <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="2" t="s">
+      <c r="A50" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D50" s="8" t="s">
+      <c r="D50" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="5"/>
+      <c r="E50" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="51" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
@@ -1448,20 +1659,24 @@
       <c r="F53" s="4"/>
     </row>
     <row r="54" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="A54" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C54" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D54" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E54" s="6"/>
-      <c r="F54" s="5"/>
+      <c r="D54" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="55" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
@@ -1488,20 +1703,24 @@
       <c r="F57" s="4"/>
     </row>
     <row r="58" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" s="2" t="s">
+      <c r="A58" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D58" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E58" s="6"/>
-      <c r="F58" s="5"/>
+      <c r="E58" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="59" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
@@ -1528,20 +1747,24 @@
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="7" t="s">
+      <c r="A62" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B62" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C62" s="2" t="s">
+      <c r="B62" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D62" s="8" t="s">
+      <c r="D62" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E62" s="6"/>
-      <c r="F62" s="5"/>
+      <c r="E62" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="63" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
@@ -1568,20 +1791,24 @@
       <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
+      <c r="A66" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B66" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C66" s="2" t="s">
+      <c r="B66" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C66" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D66" s="8" t="s">
+      <c r="D66" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E66" s="6"/>
-      <c r="F66" s="5"/>
+      <c r="E66" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="67" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
@@ -1608,20 +1835,24 @@
       <c r="F69" s="4"/>
     </row>
     <row r="70" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="7" t="s">
+      <c r="A70" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B70" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C70" s="2" t="s">
+      <c r="B70" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D70" s="8" t="s">
+      <c r="D70" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E70" s="6"/>
-      <c r="F70" s="5"/>
+      <c r="E70" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="71" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
@@ -1648,20 +1879,24 @@
       <c r="F73" s="4"/>
     </row>
     <row r="74" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="7" t="s">
+      <c r="A74" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B74" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C74" s="2" t="s">
+      <c r="B74" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C74" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D74" s="8" t="s">
+      <c r="D74" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E74" s="6"/>
-      <c r="F74" s="5"/>
+      <c r="E74" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="75" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
@@ -1688,20 +1923,24 @@
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="7" t="s">
+      <c r="A78" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B78" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C78" s="2" t="s">
+      <c r="B78" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C78" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="D78" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E78" s="6"/>
-      <c r="F78" s="5"/>
+      <c r="E78" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="79" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
@@ -1728,20 +1967,24 @@
       <c r="F81" s="4"/>
     </row>
     <row r="82" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="7" t="s">
+      <c r="A82" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B82" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E82" s="6"/>
-      <c r="F82" s="5"/>
+      <c r="B82" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="83" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
@@ -1768,20 +2011,24 @@
       <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="7" t="s">
+      <c r="A86" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B86" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E86" s="6"/>
-      <c r="F86" s="5"/>
+      <c r="B86" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="87" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
@@ -1808,20 +2055,24 @@
       <c r="F89" s="4"/>
     </row>
     <row r="90" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="7" t="s">
+      <c r="A90" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B90" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C90" s="2" t="s">
+      <c r="B90" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C90" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D90" s="8" t="s">
+      <c r="D90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E90" s="6"/>
-      <c r="F90" s="5"/>
+      <c r="E90" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="91" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
@@ -1848,20 +2099,24 @@
       <c r="F93" s="4"/>
     </row>
     <row r="94" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="7" t="s">
+      <c r="A94" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B94" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C94" s="2" t="s">
+      <c r="B94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C94" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D94" s="8" t="s">
+      <c r="D94" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E94" s="6"/>
-      <c r="F94" s="5"/>
+      <c r="E94" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="95" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
@@ -1888,20 +2143,24 @@
       <c r="F97" s="4"/>
     </row>
     <row r="98" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="7" t="s">
+      <c r="A98" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B98" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D98" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="E98" s="6"/>
-      <c r="F98" s="5"/>
+      <c r="B98" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E98" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="99" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
@@ -1928,20 +2187,24 @@
       <c r="F101" s="4"/>
     </row>
     <row r="102" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D102" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E102" s="6"/>
-      <c r="F102" s="5"/>
+      <c r="A102" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E102" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="103" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
@@ -1968,20 +2231,24 @@
       <c r="F105" s="4"/>
     </row>
     <row r="106" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D106" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="E106" s="6"/>
-      <c r="F106" s="5"/>
+      <c r="A106" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E106" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="107" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
@@ -2008,20 +2275,24 @@
       <c r="F109" s="4"/>
     </row>
     <row r="110" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D110" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="E110" s="6"/>
-      <c r="F110" s="5"/>
+      <c r="A110" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E110" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="111" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
@@ -2048,20 +2319,24 @@
       <c r="F113" s="4"/>
     </row>
     <row r="114" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D114" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="E114" s="6"/>
-      <c r="F114" s="5"/>
+      <c r="A114" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="115" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
@@ -2088,20 +2363,24 @@
       <c r="F117" s="4"/>
     </row>
     <row r="118" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D118" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="E118" s="6"/>
-      <c r="F118" s="5"/>
+      <c r="A118" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="119" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
@@ -2128,20 +2407,24 @@
       <c r="F121" s="4"/>
     </row>
     <row r="122" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D122" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E122" s="6"/>
-      <c r="F122" s="5"/>
+      <c r="A122" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D122" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E122" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="123" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
@@ -2168,20 +2451,24 @@
       <c r="F125" s="4"/>
     </row>
     <row r="126" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B126" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D126" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E126" s="6"/>
-      <c r="F126" s="5"/>
+      <c r="A126" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C126" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D126" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E126" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="127" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3"/>
@@ -2208,20 +2495,24 @@
       <c r="F129" s="4"/>
     </row>
     <row r="130" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="7" t="s">
+      <c r="A130" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C130" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B130" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C130" s="2" t="s">
+      <c r="D130" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D130" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E130" s="6"/>
-      <c r="F130" s="5"/>
+      <c r="E130" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="131" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
@@ -2248,20 +2539,24 @@
       <c r="F133" s="4"/>
     </row>
     <row r="134" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D134" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E134" s="6"/>
-      <c r="F134" s="5"/>
+      <c r="A134" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C134" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D134" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="135" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
@@ -2288,20 +2583,24 @@
       <c r="F137" s="4"/>
     </row>
     <row r="138" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D138" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E138" s="6"/>
-      <c r="F138" s="5"/>
+      <c r="A138" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C138" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D138" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="139" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3"/>
@@ -2328,20 +2627,24 @@
       <c r="F141" s="4"/>
     </row>
     <row r="142" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C142" s="2" t="s">
+      <c r="A142" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C142" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D142" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E142" s="6"/>
-      <c r="F142" s="5"/>
+      <c r="D142" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E142" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="143" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3"/>
@@ -2368,20 +2671,24 @@
       <c r="F145" s="4"/>
     </row>
     <row r="146" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="B146" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D146" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="E146" s="6"/>
-      <c r="F146" s="5"/>
+      <c r="A146" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D146" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E146" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="147" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3"/>
@@ -2408,20 +2715,24 @@
       <c r="F149" s="4"/>
     </row>
     <row r="150" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C150" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="D150" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E150" s="6"/>
-      <c r="F150" s="5"/>
+      <c r="A150" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C150" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E150" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="151" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3"/>
@@ -2448,20 +2759,24 @@
       <c r="F153" s="4"/>
     </row>
     <row r="154" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B154" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D154" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E154" s="6"/>
-      <c r="F154" s="5"/>
+      <c r="A154" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C154" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D154" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E154" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="155" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="3"/>
@@ -2488,20 +2803,24 @@
       <c r="F157" s="4"/>
     </row>
     <row r="158" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D158" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="E158" s="6"/>
-      <c r="F158" s="5"/>
+      <c r="A158" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C158" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D158" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E158" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="F158" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="159" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="3"/>
@@ -2528,20 +2847,24 @@
       <c r="F161" s="4"/>
     </row>
     <row r="162" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="B162" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C162" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D162" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="E162" s="6"/>
-      <c r="F162" s="5"/>
+      <c r="A162" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C162" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D162" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E162" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="163" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
@@ -2568,20 +2891,24 @@
       <c r="F165" s="4"/>
     </row>
     <row r="166" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="B166" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D166" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E166" s="6"/>
-      <c r="F166" s="5"/>
+      <c r="A166" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C166" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D166" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E166" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="F166" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="167" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3"/>
@@ -2608,20 +2935,24 @@
       <c r="F169" s="4"/>
     </row>
     <row r="170" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A170" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B170" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C170" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D170" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="E170" s="6"/>
-      <c r="F170" s="5"/>
+      <c r="A170" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C170" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D170" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E170" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="F170" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="171" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="3"/>
@@ -2648,20 +2979,24 @@
       <c r="F173" s="4"/>
     </row>
     <row r="174" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B174" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D174" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="E174" s="6"/>
-      <c r="F174" s="5"/>
+      <c r="A174" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C174" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D174" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E174" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="175" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="3"/>
@@ -2688,20 +3023,24 @@
       <c r="F177" s="4"/>
     </row>
     <row r="178" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B178" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C178" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D178" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="E178" s="6"/>
-      <c r="F178" s="5"/>
+      <c r="A178" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C178" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D178" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E178" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="F178" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="179" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="3"/>
@@ -2728,20 +3067,24 @@
       <c r="F181" s="4"/>
     </row>
     <row r="182" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A182" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="B182" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D182" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E182" s="6"/>
-      <c r="F182" s="5"/>
+      <c r="A182" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C182" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D182" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="F182" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="183" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="3"/>
@@ -2768,20 +3111,24 @@
       <c r="F185" s="4"/>
     </row>
     <row r="186" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="7" t="s">
+      <c r="A186" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C186" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B186" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C186" s="2" t="s">
+      <c r="D186" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D186" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="E186" s="6"/>
-      <c r="F186" s="5"/>
+      <c r="E186" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="F186" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="187" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="3"/>
@@ -2808,20 +3155,24 @@
       <c r="F189" s="4"/>
     </row>
     <row r="190" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B190" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C190" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D190" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="E190" s="6"/>
-      <c r="F190" s="5"/>
+      <c r="A190" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C190" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D190" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E190" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F190" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="191" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="3"/>
@@ -2848,20 +3199,24 @@
       <c r="F193" s="4"/>
     </row>
     <row r="194" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="B194" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C194" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="D194" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="E194" s="6"/>
-      <c r="F194" s="5"/>
+      <c r="A194" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C194" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D194" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E194" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="F194" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="195" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="3"/>
@@ -2888,20 +3243,24 @@
       <c r="F197" s="4"/>
     </row>
     <row r="198" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A198" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B198" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D198" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="E198" s="6"/>
-      <c r="F198" s="5"/>
+      <c r="A198" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C198" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D198" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E198" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="F198" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="199" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="3"/>
@@ -2929,307 +3288,308 @@
     </row>
   </sheetData>
   <mergeCells count="300">
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="B2:B5"/>
     <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="C150:C153"/>
-    <mergeCell ref="C190:C193"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B29"/>
     <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="E26:E29"/>
     <mergeCell ref="F38:F41"/>
     <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="A74:A77"/>
     <mergeCell ref="B74:B77"/>
-    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="F110:F113"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="C150:C153"/>
+    <mergeCell ref="D150:D153"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="D162:D165"/>
     <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="B158:B161"/>
     <mergeCell ref="C158:C161"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="D166:D169"/>
     <mergeCell ref="E166:E169"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D174:D177"/>
     <mergeCell ref="F174:F177"/>
     <mergeCell ref="A178:A181"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="F110:F113"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="E190:E193"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update test cases Excel file with new test scenarios
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mandini\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yasith Lakruwan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8608379-8882-40FC-A87B-B4999CD81ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C24CB8A3-34FD-40A6-B78B-181225D6BCCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="287">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -647,6 +647,244 @@
   </si>
   <si>
     <t>පොඩ්ඩක් මේ website එක බලන්න : https://www.ස්ලිත්ම්.ඇඩු.ල්ක්/</t>
+  </si>
+  <si>
+    <t>Singlish input types covered</t>
+  </si>
+  <si>
+    <t>Evidence / Rationale</t>
+  </si>
+  <si>
+    <t>Question forms</t>
+  </si>
+  <si>
+    <t>Command forms</t>
+  </si>
+  <si>
+    <t>Greetings</t>
+  </si>
+  <si>
+    <t>Rationale: The sentence is a question ending with “keeyda?”.
+Evidence: The word “litr” represents a measurement unit (liter) written in Singlish.</t>
+  </si>
+  <si>
+    <t>Rationale: The phrase asks a question using “giyda?”.
+Evidence: The term “keeyk” expresses a numeric quantity in Singlish form.</t>
+  </si>
+  <si>
+    <t>Evidence: The verb “denna” is used as a direct instruction.</t>
+  </si>
+  <si>
+    <t>Evidence: “karunakarala” indicates a polite request.
+Rationale: A comma is used within the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: The phrase begins with “suba udasanak”, a common Sinhala greeting.</t>
+  </si>
+  <si>
+    <t>Evidence: The sentence conveys well-wishing using “suba pathum”.</t>
+  </si>
+  <si>
+    <t>Evidence: The phrase “puluwannam” is used to make a request politely.</t>
+  </si>
+  <si>
+    <t>Evidence: The word “gennako” expresses a casual request.</t>
+  </si>
+  <si>
+    <t>Evidence: The word “hari” is used as a response.
+Rationale: A comma is used as punctuation.</t>
+  </si>
+  <si>
+    <t>Evidence: “litr” is a unit of measurement and “10i” expresses numeric style.</t>
+  </si>
+  <si>
+    <t>Evidence: The word “pata” is repeated consecutively.</t>
+  </si>
+  <si>
+    <t>Evidence: The sound word “hu hu” is intentionally repeated.</t>
+  </si>
+  <si>
+    <t>Evidence: Quotation marks are used in the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: The sentence is enclosed in quotation marks.</t>
+  </si>
+  <si>
+    <t>Evidence: Words like “mm” and “withrai” show non-standard Singlish spellings.</t>
+  </si>
+  <si>
+    <t>Evidence: Variants like “mn”, “kagahuwa”, “kaghnwa” show inconsistent spelling.</t>
+  </si>
+  <si>
+    <t>Evidence: The single English word “work” is inserted between Singlish words.</t>
+  </si>
+  <si>
+    <t>Evidence: The English word “yoghurt” is inserted into Singlish text.</t>
+  </si>
+  <si>
+    <t>Evidence: The phrase “bike eke” combines English and Singlish words as a phrase.</t>
+  </si>
+  <si>
+    <t>Evidence: The phrase “official work” appears as consecutive English words.</t>
+  </si>
+  <si>
+    <t>Evidence: The digital term “log” is used within Singlish.</t>
+  </si>
+  <si>
+    <t>Evidence: Digital terms “git” and “pull” are embedded in the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: The platform name “eduscope” is directly used.</t>
+  </si>
+  <si>
+    <t>Evidence: The app name “temu” is included in the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: Acronyms “vm” and “dns” are used.</t>
+  </si>
+  <si>
+    <t>Evidence: The acronym “smtp” appears in the input.</t>
+  </si>
+  <si>
+    <t>Evidence: The clipped English word “pitch” is used.</t>
+  </si>
+  <si>
+    <t>Evidence: The clipped form “race” is used within Singlish.</t>
+  </si>
+  <si>
+    <t>Evidence: The place name “Switzerland” is embedded in the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: The place name “Vietnam” is used.</t>
+  </si>
+  <si>
+    <t>Evidence: The person name “Kohli” is included.</t>
+  </si>
+  <si>
+    <t>Evidence: The personal name “Sachithra” appears in the sentence.</t>
+  </si>
+  <si>
+    <t>Evidence: “4th gen” shows numeric suffix usage.</t>
+  </si>
+  <si>
+    <t>Evidence: “6k”, “3k” are numeric suffix forms.</t>
+  </si>
+  <si>
+    <t>Evidence: “100k” represents money in numeric currency style.</t>
+  </si>
+  <si>
+    <t>Evidence: The term “riyal” represents a currency name.</t>
+  </si>
+  <si>
+    <t>Evidence: “9.30 a.m.” is a time format.</t>
+  </si>
+  <si>
+    <t>Evidence: “10.00a.m.” is a time format.</t>
+  </si>
+  <si>
+    <t>Evidence: The date “June 7” appears in the input.</t>
+  </si>
+  <si>
+    <t>Evidence: The date “May 30” is included.</t>
+  </si>
+  <si>
+    <t>Evidence: “litr 1000k” represents measurement with numeric suffix.</t>
+  </si>
+  <si>
+    <t>Evidence: “kilomitr 130k” shows a measurement unit.</t>
+  </si>
+  <si>
+    <t>Evidence: Slang terms like “mchn”, “elakirine” are used.</t>
+  </si>
+  <si>
+    <t>Evidence: Casual slang words like “dial”, “bn” appear.</t>
+  </si>
+  <si>
+    <t>Evidence: A URL starting with “https://” is present.</t>
+  </si>
+  <si>
+    <t>Evidence: An email address is included.</t>
+  </si>
+  <si>
+    <t>Evidence: The emoji 😡 is present in the input.</t>
+  </si>
+  <si>
+    <t>Evidence: The emoji 🥰 is included.</t>
+  </si>
+  <si>
+    <t>Evidence: Words like “tikk”, “amru” show informal spelling variants.</t>
+  </si>
+  <si>
+    <t>Evidence: Words like “eylat”, “paren” show non-standard Singlish spelling.</t>
+  </si>
+  <si>
+    <t>Requests</t>
+  </si>
+  <si>
+    <t>Responses</t>
+  </si>
+  <si>
+    <t>Repeated Words</t>
+  </si>
+  <si>
+    <t>Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t>Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t>Multi-Word English Phrases in Singlish</t>
+  </si>
+  <si>
+    <t>English Digital Terms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Platform/App Names in Singlish</t>
+  </si>
+  <si>
+    <t>English Abbreviations/Acronyms in Singlish</t>
+  </si>
+  <si>
+    <t>English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t>Place Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Person Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Inputs with Numbers and Numeric Suffixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Inputs with Currency</t>
+  </si>
+  <si>
+    <t>Inputs with Time Formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs with Dates </t>
+  </si>
+  <si>
+    <t>Inputs with Unit of Measurements</t>
+  </si>
+  <si>
+    <t>Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t>Online Indentifiers in Singlish</t>
+  </si>
+  <si>
+    <t>Inputs Containing Emojis</t>
+  </si>
+  <si>
+    <t>singlish</t>
+  </si>
+  <si>
+    <t>Singlish</t>
   </si>
 </sst>
 </file>
@@ -701,7 +939,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -748,11 +986,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -774,6 +1025,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1054,19 +1317,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr defaultRowHeight="49.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
     <col min="3" max="3" width="22.140625" customWidth="1"/>
     <col min="4" max="4" width="25.28515625" customWidth="1"/>
     <col min="5" max="5" width="22.5703125" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="10" width="12.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.140625" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="13" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1085,8 +1350,15 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="I1" s="9"/>
+    </row>
+    <row r="2" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -1105,32 +1377,48 @@
       <c r="F2" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="I2" s="10"/>
+    </row>
+    <row r="3" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="10"/>
+    </row>
+    <row r="4" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="10"/>
+    </row>
+    <row r="5" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-    </row>
-    <row r="6" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="10"/>
+    </row>
+    <row r="6" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
@@ -1149,32 +1437,48 @@
       <c r="F6" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G6" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I6" s="10"/>
+    </row>
+    <row r="7" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1193,32 +1497,48 @@
       <c r="F10" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G10" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="I10" s="10"/>
+    </row>
+    <row r="11" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-    </row>
-    <row r="13" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -1237,32 +1557,48 @@
       <c r="F14" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="I14" s="10"/>
+    </row>
+    <row r="15" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-    </row>
-    <row r="17" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
@@ -1281,32 +1617,48 @@
       <c r="F18" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="I18" s="10"/>
+    </row>
+    <row r="19" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
-    </row>
-    <row r="20" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-    </row>
-    <row r="21" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>22</v>
       </c>
@@ -1325,32 +1677,48 @@
       <c r="F22" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G22" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="I22" s="10"/>
+    </row>
+    <row r="23" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
-    </row>
-    <row r="24" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-    </row>
-    <row r="25" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
-    </row>
-    <row r="26" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>25</v>
       </c>
@@ -1369,32 +1737,48 @@
       <c r="F26" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G26" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="I26" s="10"/>
+    </row>
+    <row r="27" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
-    </row>
-    <row r="28" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
-    </row>
-    <row r="29" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="11"/>
+    </row>
+    <row r="29" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
-    </row>
-    <row r="30" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="11"/>
+    </row>
+    <row r="30" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>28</v>
       </c>
@@ -1413,32 +1797,48 @@
       <c r="F30" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G30" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="I30" s="10"/>
+    </row>
+    <row r="31" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="11"/>
+    </row>
+    <row r="32" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-    </row>
-    <row r="34" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>31</v>
       </c>
@@ -1457,32 +1857,48 @@
       <c r="F34" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G34" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="I34" s="10"/>
+    </row>
+    <row r="35" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
-    </row>
-    <row r="36" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
-    </row>
-    <row r="37" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
-    </row>
-    <row r="38" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>34</v>
       </c>
@@ -1501,32 +1917,48 @@
       <c r="F38" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G38" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="I38" s="10"/>
+    </row>
+    <row r="39" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
-    </row>
-    <row r="40" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
-    </row>
-    <row r="41" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G40" s="13"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="11"/>
+    </row>
+    <row r="41" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
-    </row>
-    <row r="42" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="11"/>
+    </row>
+    <row r="42" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>37</v>
       </c>
@@ -1545,32 +1977,48 @@
       <c r="F42" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G42" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="I42" s="10"/>
+    </row>
+    <row r="43" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
-    </row>
-    <row r="44" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="11"/>
+    </row>
+    <row r="44" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
-    </row>
-    <row r="45" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="11"/>
+    </row>
+    <row r="45" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
-    </row>
-    <row r="46" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="11"/>
+    </row>
+    <row r="46" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>40</v>
       </c>
@@ -1589,32 +2037,48 @@
       <c r="F46" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G46" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="I46" s="10"/>
+    </row>
+    <row r="47" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
-    </row>
-    <row r="48" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G47" s="13"/>
+      <c r="H47" s="13"/>
+      <c r="I47" s="11"/>
+    </row>
+    <row r="48" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
-    </row>
-    <row r="49" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G48" s="13"/>
+      <c r="H48" s="13"/>
+      <c r="I48" s="11"/>
+    </row>
+    <row r="49" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
-    </row>
-    <row r="50" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="11"/>
+    </row>
+    <row r="50" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>43</v>
       </c>
@@ -1633,32 +2097,48 @@
       <c r="F50" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G50" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="I50" s="10"/>
+    </row>
+    <row r="51" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
-    </row>
-    <row r="52" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="11"/>
+    </row>
+    <row r="52" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
-    </row>
-    <row r="53" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G52" s="13"/>
+      <c r="H52" s="13"/>
+      <c r="I52" s="11"/>
+    </row>
+    <row r="53" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
-    </row>
-    <row r="54" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="11"/>
+    </row>
+    <row r="54" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>44</v>
       </c>
@@ -1677,32 +2157,48 @@
       <c r="F54" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G54" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="I54" s="10"/>
+    </row>
+    <row r="55" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
-    </row>
-    <row r="56" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="11"/>
+    </row>
+    <row r="56" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
-    </row>
-    <row r="57" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
-    </row>
-    <row r="58" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G57" s="14"/>
+      <c r="H57" s="14"/>
+      <c r="I57" s="11"/>
+    </row>
+    <row r="58" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>47</v>
       </c>
@@ -1721,32 +2217,48 @@
       <c r="F58" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G58" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="H58" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="I58" s="10"/>
+    </row>
+    <row r="59" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
-    </row>
-    <row r="60" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G59" s="13"/>
+      <c r="H59" s="13"/>
+      <c r="I59" s="11"/>
+    </row>
+    <row r="60" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
-    </row>
-    <row r="61" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G60" s="13"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="11"/>
+    </row>
+    <row r="61" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
-    </row>
-    <row r="62" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G61" s="14"/>
+      <c r="H61" s="14"/>
+      <c r="I61" s="11"/>
+    </row>
+    <row r="62" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>53</v>
       </c>
@@ -1765,32 +2277,48 @@
       <c r="F62" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G62" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="H62" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="I62" s="10"/>
+    </row>
+    <row r="63" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
-    </row>
-    <row r="64" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G63" s="13"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="11"/>
+    </row>
+    <row r="64" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
-    </row>
-    <row r="65" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G64" s="13"/>
+      <c r="H64" s="13"/>
+      <c r="I64" s="11"/>
+    </row>
+    <row r="65" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
-    </row>
-    <row r="66" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G65" s="14"/>
+      <c r="H65" s="14"/>
+      <c r="I65" s="11"/>
+    </row>
+    <row r="66" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>56</v>
       </c>
@@ -1809,32 +2337,48 @@
       <c r="F66" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G66" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="H66" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="I66" s="10"/>
+    </row>
+    <row r="67" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
-    </row>
-    <row r="68" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="11"/>
+    </row>
+    <row r="68" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
-    </row>
-    <row r="69" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G68" s="13"/>
+      <c r="H68" s="13"/>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
-    </row>
-    <row r="70" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G69" s="14"/>
+      <c r="H69" s="14"/>
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>59</v>
       </c>
@@ -1853,32 +2397,48 @@
       <c r="F70" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G70" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="H70" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="I70" s="10"/>
+    </row>
+    <row r="71" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
-    </row>
-    <row r="72" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G71" s="13"/>
+      <c r="H71" s="13"/>
+      <c r="I71" s="11"/>
+    </row>
+    <row r="72" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
-    </row>
-    <row r="73" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G72" s="13"/>
+      <c r="H72" s="13"/>
+      <c r="I72" s="11"/>
+    </row>
+    <row r="73" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
-    </row>
-    <row r="74" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G73" s="14"/>
+      <c r="H73" s="14"/>
+      <c r="I73" s="11"/>
+    </row>
+    <row r="74" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>62</v>
       </c>
@@ -1897,32 +2457,48 @@
       <c r="F74" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G74" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="H74" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="I74" s="10"/>
+    </row>
+    <row r="75" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
-    </row>
-    <row r="76" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G75" s="13"/>
+      <c r="H75" s="13"/>
+      <c r="I75" s="11"/>
+    </row>
+    <row r="76" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
-    </row>
-    <row r="77" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G76" s="13"/>
+      <c r="H76" s="13"/>
+      <c r="I76" s="11"/>
+    </row>
+    <row r="77" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
-    </row>
-    <row r="78" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G77" s="14"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="11"/>
+    </row>
+    <row r="78" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>65</v>
       </c>
@@ -1941,32 +2517,48 @@
       <c r="F78" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G78" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="H78" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="I78" s="10"/>
+    </row>
+    <row r="79" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
-    </row>
-    <row r="80" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G79" s="13"/>
+      <c r="H79" s="13"/>
+      <c r="I79" s="11"/>
+    </row>
+    <row r="80" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
-    </row>
-    <row r="81" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G80" s="13"/>
+      <c r="H80" s="13"/>
+      <c r="I80" s="11"/>
+    </row>
+    <row r="81" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4"/>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
       <c r="D81" s="4"/>
       <c r="E81" s="4"/>
       <c r="F81" s="4"/>
-    </row>
-    <row r="82" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G81" s="14"/>
+      <c r="H81" s="14"/>
+      <c r="I81" s="11"/>
+    </row>
+    <row r="82" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>68</v>
       </c>
@@ -1985,32 +2577,48 @@
       <c r="F82" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G82" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="H82" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="I82" s="10"/>
+    </row>
+    <row r="83" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
-    </row>
-    <row r="84" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G83" s="13"/>
+      <c r="H83" s="13"/>
+      <c r="I83" s="11"/>
+    </row>
+    <row r="84" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
-    </row>
-    <row r="85" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G84" s="13"/>
+      <c r="H84" s="13"/>
+      <c r="I84" s="11"/>
+    </row>
+    <row r="85" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4"/>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
       <c r="D85" s="4"/>
       <c r="E85" s="4"/>
       <c r="F85" s="4"/>
-    </row>
-    <row r="86" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G85" s="14"/>
+      <c r="H85" s="14"/>
+      <c r="I85" s="11"/>
+    </row>
+    <row r="86" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>71</v>
       </c>
@@ -2029,32 +2637,48 @@
       <c r="F86" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G86" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="H86" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="I86" s="10"/>
+    </row>
+    <row r="87" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
-    </row>
-    <row r="88" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G87" s="13"/>
+      <c r="H87" s="13"/>
+      <c r="I87" s="11"/>
+    </row>
+    <row r="88" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
-    </row>
-    <row r="89" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G88" s="13"/>
+      <c r="H88" s="13"/>
+      <c r="I88" s="11"/>
+    </row>
+    <row r="89" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4"/>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
       <c r="D89" s="4"/>
       <c r="E89" s="4"/>
       <c r="F89" s="4"/>
-    </row>
-    <row r="90" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G89" s="14"/>
+      <c r="H89" s="14"/>
+      <c r="I89" s="11"/>
+    </row>
+    <row r="90" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
         <v>74</v>
       </c>
@@ -2073,32 +2697,48 @@
       <c r="F90" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G90" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="H90" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="I90" s="10"/>
+    </row>
+    <row r="91" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
-    </row>
-    <row r="92" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G91" s="13"/>
+      <c r="H91" s="13"/>
+      <c r="I91" s="11"/>
+    </row>
+    <row r="92" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
-    </row>
-    <row r="93" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G92" s="13"/>
+      <c r="H92" s="13"/>
+      <c r="I92" s="11"/>
+    </row>
+    <row r="93" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
       <c r="F93" s="4"/>
-    </row>
-    <row r="94" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G93" s="14"/>
+      <c r="H93" s="14"/>
+      <c r="I93" s="11"/>
+    </row>
+    <row r="94" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>77</v>
       </c>
@@ -2117,32 +2757,48 @@
       <c r="F94" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G94" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="H94" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="I94" s="10"/>
+    </row>
+    <row r="95" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
-    </row>
-    <row r="96" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G95" s="13"/>
+      <c r="H95" s="13"/>
+      <c r="I95" s="11"/>
+    </row>
+    <row r="96" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
-    </row>
-    <row r="97" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G96" s="13"/>
+      <c r="H96" s="13"/>
+      <c r="I96" s="11"/>
+    </row>
+    <row r="97" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
       <c r="F97" s="4"/>
-    </row>
-    <row r="98" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G97" s="14"/>
+      <c r="H97" s="14"/>
+      <c r="I97" s="11"/>
+    </row>
+    <row r="98" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>80</v>
       </c>
@@ -2161,32 +2817,48 @@
       <c r="F98" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G98" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="H98" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="I98" s="10"/>
+    </row>
+    <row r="99" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
-    </row>
-    <row r="100" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G99" s="13"/>
+      <c r="H99" s="13"/>
+      <c r="I99" s="11"/>
+    </row>
+    <row r="100" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
-    </row>
-    <row r="101" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G100" s="13"/>
+      <c r="H100" s="13"/>
+      <c r="I100" s="11"/>
+    </row>
+    <row r="101" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
       <c r="F101" s="4"/>
-    </row>
-    <row r="102" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G101" s="14"/>
+      <c r="H101" s="14"/>
+      <c r="I101" s="11"/>
+    </row>
+    <row r="102" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>81</v>
       </c>
@@ -2205,32 +2877,48 @@
       <c r="F102" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G102" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="H102" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="I102" s="10"/>
+    </row>
+    <row r="103" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
-    </row>
-    <row r="104" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G103" s="13"/>
+      <c r="H103" s="13"/>
+      <c r="I103" s="11"/>
+    </row>
+    <row r="104" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
-    </row>
-    <row r="105" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G104" s="13"/>
+      <c r="H104" s="13"/>
+      <c r="I104" s="11"/>
+    </row>
+    <row r="105" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
       <c r="D105" s="4"/>
       <c r="E105" s="4"/>
       <c r="F105" s="4"/>
-    </row>
-    <row r="106" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G105" s="14"/>
+      <c r="H105" s="14"/>
+      <c r="I105" s="11"/>
+    </row>
+    <row r="106" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
         <v>82</v>
       </c>
@@ -2249,32 +2937,48 @@
       <c r="F106" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G106" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="H106" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="I106" s="10"/>
+    </row>
+    <row r="107" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
       <c r="F107" s="3"/>
-    </row>
-    <row r="108" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G107" s="13"/>
+      <c r="H107" s="13"/>
+      <c r="I107" s="11"/>
+    </row>
+    <row r="108" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
       <c r="F108" s="3"/>
-    </row>
-    <row r="109" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G108" s="13"/>
+      <c r="H108" s="13"/>
+      <c r="I108" s="11"/>
+    </row>
+    <row r="109" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="4"/>
-    </row>
-    <row r="110" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G109" s="14"/>
+      <c r="H109" s="14"/>
+      <c r="I109" s="11"/>
+    </row>
+    <row r="110" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
         <v>85</v>
       </c>
@@ -2293,32 +2997,48 @@
       <c r="F110" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G110" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="H110" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="I110" s="10"/>
+    </row>
+    <row r="111" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
       <c r="F111" s="3"/>
-    </row>
-    <row r="112" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G111" s="13"/>
+      <c r="H111" s="13"/>
+      <c r="I111" s="11"/>
+    </row>
+    <row r="112" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
       <c r="F112" s="3"/>
-    </row>
-    <row r="113" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G112" s="13"/>
+      <c r="H112" s="13"/>
+      <c r="I112" s="11"/>
+    </row>
+    <row r="113" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="4"/>
-    </row>
-    <row r="114" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G113" s="14"/>
+      <c r="H113" s="14"/>
+      <c r="I113" s="11"/>
+    </row>
+    <row r="114" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
         <v>88</v>
       </c>
@@ -2337,32 +3057,48 @@
       <c r="F114" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G114" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="H114" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="I114" s="10"/>
+    </row>
+    <row r="115" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
       <c r="F115" s="3"/>
-    </row>
-    <row r="116" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G115" s="13"/>
+      <c r="H115" s="13"/>
+      <c r="I115" s="11"/>
+    </row>
+    <row r="116" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
       <c r="F116" s="3"/>
-    </row>
-    <row r="117" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G116" s="13"/>
+      <c r="H116" s="13"/>
+      <c r="I116" s="11"/>
+    </row>
+    <row r="117" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="4"/>
-    </row>
-    <row r="118" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G117" s="14"/>
+      <c r="H117" s="14"/>
+      <c r="I117" s="11"/>
+    </row>
+    <row r="118" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
         <v>91</v>
       </c>
@@ -2381,32 +3117,48 @@
       <c r="F118" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G118" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="H118" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="I118" s="10"/>
+    </row>
+    <row r="119" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
       <c r="F119" s="3"/>
-    </row>
-    <row r="120" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G119" s="13"/>
+      <c r="H119" s="13"/>
+      <c r="I119" s="11"/>
+    </row>
+    <row r="120" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
       <c r="F120" s="3"/>
-    </row>
-    <row r="121" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G120" s="13"/>
+      <c r="H120" s="13"/>
+      <c r="I120" s="11"/>
+    </row>
+    <row r="121" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
       <c r="D121" s="4"/>
       <c r="E121" s="4"/>
       <c r="F121" s="4"/>
-    </row>
-    <row r="122" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G121" s="14"/>
+      <c r="H121" s="14"/>
+      <c r="I121" s="11"/>
+    </row>
+    <row r="122" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
         <v>94</v>
       </c>
@@ -2425,32 +3177,48 @@
       <c r="F122" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G122" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="H122" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="I122" s="10"/>
+    </row>
+    <row r="123" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
       <c r="F123" s="3"/>
-    </row>
-    <row r="124" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G123" s="13"/>
+      <c r="H123" s="13"/>
+      <c r="I123" s="11"/>
+    </row>
+    <row r="124" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
       <c r="F124" s="3"/>
-    </row>
-    <row r="125" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G124" s="13"/>
+      <c r="H124" s="13"/>
+      <c r="I124" s="11"/>
+    </row>
+    <row r="125" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
       <c r="F125" s="4"/>
-    </row>
-    <row r="126" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G125" s="14"/>
+      <c r="H125" s="14"/>
+      <c r="I125" s="11"/>
+    </row>
+    <row r="126" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
         <v>97</v>
       </c>
@@ -2469,32 +3237,48 @@
       <c r="F126" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="127" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G126" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="H126" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="I126" s="10"/>
+    </row>
+    <row r="127" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
       <c r="F127" s="3"/>
-    </row>
-    <row r="128" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G127" s="13"/>
+      <c r="H127" s="13"/>
+      <c r="I127" s="11"/>
+    </row>
+    <row r="128" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
       <c r="D128" s="3"/>
       <c r="E128" s="3"/>
       <c r="F128" s="3"/>
-    </row>
-    <row r="129" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G128" s="13"/>
+      <c r="H128" s="13"/>
+      <c r="I128" s="11"/>
+    </row>
+    <row r="129" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4"/>
-    </row>
-    <row r="130" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G129" s="14"/>
+      <c r="H129" s="14"/>
+      <c r="I129" s="11"/>
+    </row>
+    <row r="130" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
         <v>100</v>
       </c>
@@ -2513,32 +3297,48 @@
       <c r="F130" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G130" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="H130" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="I130" s="10"/>
+    </row>
+    <row r="131" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="E131" s="3"/>
       <c r="F131" s="3"/>
-    </row>
-    <row r="132" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G131" s="13"/>
+      <c r="H131" s="13"/>
+      <c r="I131" s="11"/>
+    </row>
+    <row r="132" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="3"/>
       <c r="F132" s="3"/>
-    </row>
-    <row r="133" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G132" s="13"/>
+      <c r="H132" s="13"/>
+      <c r="I132" s="11"/>
+    </row>
+    <row r="133" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="4"/>
       <c r="D133" s="4"/>
       <c r="E133" s="4"/>
       <c r="F133" s="4"/>
-    </row>
-    <row r="134" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G133" s="14"/>
+      <c r="H133" s="14"/>
+      <c r="I133" s="11"/>
+    </row>
+    <row r="134" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
         <v>101</v>
       </c>
@@ -2557,32 +3357,48 @@
       <c r="F134" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G134" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="H134" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="I134" s="10"/>
+    </row>
+    <row r="135" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="3"/>
       <c r="F135" s="3"/>
-    </row>
-    <row r="136" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G135" s="13"/>
+      <c r="H135" s="13"/>
+      <c r="I135" s="11"/>
+    </row>
+    <row r="136" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="E136" s="3"/>
       <c r="F136" s="3"/>
-    </row>
-    <row r="137" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G136" s="13"/>
+      <c r="H136" s="13"/>
+      <c r="I136" s="11"/>
+    </row>
+    <row r="137" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" s="4"/>
       <c r="D137" s="4"/>
       <c r="E137" s="4"/>
       <c r="F137" s="4"/>
-    </row>
-    <row r="138" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G137" s="14"/>
+      <c r="H137" s="14"/>
+      <c r="I137" s="11"/>
+    </row>
+    <row r="138" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
         <v>106</v>
       </c>
@@ -2601,32 +3417,48 @@
       <c r="F138" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G138" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="H138" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="I138" s="10"/>
+    </row>
+    <row r="139" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
       <c r="D139" s="3"/>
       <c r="E139" s="3"/>
       <c r="F139" s="3"/>
-    </row>
-    <row r="140" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G139" s="13"/>
+      <c r="H139" s="13"/>
+      <c r="I139" s="11"/>
+    </row>
+    <row r="140" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
       <c r="D140" s="3"/>
       <c r="E140" s="3"/>
       <c r="F140" s="3"/>
-    </row>
-    <row r="141" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G140" s="13"/>
+      <c r="H140" s="13"/>
+      <c r="I140" s="11"/>
+    </row>
+    <row r="141" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" s="4"/>
       <c r="D141" s="4"/>
       <c r="E141" s="4"/>
       <c r="F141" s="4"/>
-    </row>
-    <row r="142" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G141" s="14"/>
+      <c r="H141" s="14"/>
+      <c r="I141" s="11"/>
+    </row>
+    <row r="142" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
         <v>109</v>
       </c>
@@ -2645,32 +3477,48 @@
       <c r="F142" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="143" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G142" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="H142" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="I142" s="10"/>
+    </row>
+    <row r="143" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
       <c r="D143" s="3"/>
       <c r="E143" s="3"/>
       <c r="F143" s="3"/>
-    </row>
-    <row r="144" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G143" s="13"/>
+      <c r="H143" s="13"/>
+      <c r="I143" s="11"/>
+    </row>
+    <row r="144" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
       <c r="F144" s="3"/>
-    </row>
-    <row r="145" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G144" s="13"/>
+      <c r="H144" s="13"/>
+      <c r="I144" s="11"/>
+    </row>
+    <row r="145" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="4"/>
       <c r="B145" s="4"/>
       <c r="C145" s="4"/>
       <c r="D145" s="4"/>
       <c r="E145" s="4"/>
       <c r="F145" s="4"/>
-    </row>
-    <row r="146" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G145" s="14"/>
+      <c r="H145" s="14"/>
+      <c r="I145" s="11"/>
+    </row>
+    <row r="146" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
         <v>110</v>
       </c>
@@ -2689,32 +3537,48 @@
       <c r="F146" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="147" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G146" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="H146" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="I146" s="10"/>
+    </row>
+    <row r="147" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
       <c r="D147" s="3"/>
       <c r="E147" s="3"/>
       <c r="F147" s="3"/>
-    </row>
-    <row r="148" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G147" s="13"/>
+      <c r="H147" s="13"/>
+      <c r="I147" s="11"/>
+    </row>
+    <row r="148" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
       <c r="E148" s="3"/>
       <c r="F148" s="3"/>
-    </row>
-    <row r="149" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G148" s="13"/>
+      <c r="H148" s="13"/>
+      <c r="I148" s="11"/>
+    </row>
+    <row r="149" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4"/>
       <c r="B149" s="4"/>
       <c r="C149" s="4"/>
       <c r="D149" s="4"/>
       <c r="E149" s="4"/>
       <c r="F149" s="4"/>
-    </row>
-    <row r="150" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G149" s="14"/>
+      <c r="H149" s="14"/>
+      <c r="I149" s="11"/>
+    </row>
+    <row r="150" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
         <v>113</v>
       </c>
@@ -2733,32 +3597,48 @@
       <c r="F150" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="151" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G150" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="H150" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="I150" s="10"/>
+    </row>
+    <row r="151" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
       <c r="D151" s="3"/>
       <c r="E151" s="3"/>
       <c r="F151" s="3"/>
-    </row>
-    <row r="152" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G151" s="13"/>
+      <c r="H151" s="13"/>
+      <c r="I151" s="11"/>
+    </row>
+    <row r="152" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
       <c r="D152" s="3"/>
       <c r="E152" s="3"/>
       <c r="F152" s="3"/>
-    </row>
-    <row r="153" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G152" s="13"/>
+      <c r="H152" s="13"/>
+      <c r="I152" s="11"/>
+    </row>
+    <row r="153" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="4"/>
       <c r="B153" s="4"/>
       <c r="C153" s="4"/>
       <c r="D153" s="4"/>
       <c r="E153" s="4"/>
       <c r="F153" s="4"/>
-    </row>
-    <row r="154" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G153" s="14"/>
+      <c r="H153" s="14"/>
+      <c r="I153" s="11"/>
+    </row>
+    <row r="154" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5" t="s">
         <v>117</v>
       </c>
@@ -2777,32 +3657,48 @@
       <c r="F154" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="155" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G154" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="H154" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="I154" s="10"/>
+    </row>
+    <row r="155" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
       <c r="E155" s="3"/>
       <c r="F155" s="3"/>
-    </row>
-    <row r="156" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G155" s="13"/>
+      <c r="H155" s="13"/>
+      <c r="I155" s="11"/>
+    </row>
+    <row r="156" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
       <c r="E156" s="3"/>
       <c r="F156" s="3"/>
-    </row>
-    <row r="157" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G156" s="13"/>
+      <c r="H156" s="13"/>
+      <c r="I156" s="11"/>
+    </row>
+    <row r="157" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="4"/>
       <c r="B157" s="4"/>
       <c r="C157" s="4"/>
       <c r="D157" s="4"/>
       <c r="E157" s="4"/>
       <c r="F157" s="4"/>
-    </row>
-    <row r="158" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G157" s="14"/>
+      <c r="H157" s="14"/>
+      <c r="I157" s="11"/>
+    </row>
+    <row r="158" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="5" t="s">
         <v>120</v>
       </c>
@@ -2821,32 +3717,48 @@
       <c r="F158" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="159" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G158" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="H158" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="I158" s="10"/>
+    </row>
+    <row r="159" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
       <c r="D159" s="3"/>
       <c r="E159" s="3"/>
       <c r="F159" s="3"/>
-    </row>
-    <row r="160" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G159" s="13"/>
+      <c r="H159" s="13"/>
+      <c r="I159" s="11"/>
+    </row>
+    <row r="160" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
       <c r="D160" s="3"/>
       <c r="E160" s="3"/>
       <c r="F160" s="3"/>
-    </row>
-    <row r="161" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G160" s="13"/>
+      <c r="H160" s="13"/>
+      <c r="I160" s="11"/>
+    </row>
+    <row r="161" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="4"/>
       <c r="B161" s="4"/>
       <c r="C161" s="4"/>
       <c r="D161" s="4"/>
       <c r="E161" s="4"/>
       <c r="F161" s="4"/>
-    </row>
-    <row r="162" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G161" s="14"/>
+      <c r="H161" s="14"/>
+      <c r="I161" s="11"/>
+    </row>
+    <row r="162" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="5" t="s">
         <v>123</v>
       </c>
@@ -2865,32 +3777,48 @@
       <c r="F162" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="163" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G162" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="H162" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="I162" s="10"/>
+    </row>
+    <row r="163" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
       <c r="D163" s="3"/>
       <c r="E163" s="3"/>
       <c r="F163" s="3"/>
-    </row>
-    <row r="164" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G163" s="13"/>
+      <c r="H163" s="13"/>
+      <c r="I163" s="11"/>
+    </row>
+    <row r="164" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
       <c r="D164" s="3"/>
       <c r="E164" s="3"/>
       <c r="F164" s="3"/>
-    </row>
-    <row r="165" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G164" s="13"/>
+      <c r="H164" s="13"/>
+      <c r="I164" s="11"/>
+    </row>
+    <row r="165" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="4"/>
       <c r="B165" s="4"/>
       <c r="C165" s="4"/>
       <c r="D165" s="4"/>
       <c r="E165" s="4"/>
       <c r="F165" s="4"/>
-    </row>
-    <row r="166" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G165" s="14"/>
+      <c r="H165" s="14"/>
+      <c r="I165" s="11"/>
+    </row>
+    <row r="166" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>126</v>
       </c>
@@ -2909,32 +3837,48 @@
       <c r="F166" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="167" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G166" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="H166" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="I166" s="10"/>
+    </row>
+    <row r="167" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
       <c r="E167" s="3"/>
       <c r="F167" s="3"/>
-    </row>
-    <row r="168" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G167" s="13"/>
+      <c r="H167" s="13"/>
+      <c r="I167" s="11"/>
+    </row>
+    <row r="168" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
       <c r="D168" s="3"/>
       <c r="E168" s="3"/>
       <c r="F168" s="3"/>
-    </row>
-    <row r="169" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G168" s="13"/>
+      <c r="H168" s="13"/>
+      <c r="I168" s="11"/>
+    </row>
+    <row r="169" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="4"/>
       <c r="B169" s="4"/>
       <c r="C169" s="4"/>
       <c r="D169" s="4"/>
       <c r="E169" s="4"/>
       <c r="F169" s="4"/>
-    </row>
-    <row r="170" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G169" s="14"/>
+      <c r="H169" s="14"/>
+      <c r="I169" s="11"/>
+    </row>
+    <row r="170" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="5" t="s">
         <v>127</v>
       </c>
@@ -2953,32 +3897,48 @@
       <c r="F170" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="171" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G170" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="H170" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="I170" s="10"/>
+    </row>
+    <row r="171" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
       <c r="D171" s="3"/>
       <c r="E171" s="3"/>
       <c r="F171" s="3"/>
-    </row>
-    <row r="172" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G171" s="13"/>
+      <c r="H171" s="13"/>
+      <c r="I171" s="11"/>
+    </row>
+    <row r="172" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
       <c r="E172" s="3"/>
       <c r="F172" s="3"/>
-    </row>
-    <row r="173" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G172" s="13"/>
+      <c r="H172" s="13"/>
+      <c r="I172" s="11"/>
+    </row>
+    <row r="173" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="4"/>
       <c r="B173" s="4"/>
       <c r="C173" s="4"/>
       <c r="D173" s="4"/>
       <c r="E173" s="4"/>
       <c r="F173" s="4"/>
-    </row>
-    <row r="174" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G173" s="14"/>
+      <c r="H173" s="14"/>
+      <c r="I173" s="11"/>
+    </row>
+    <row r="174" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="5" t="s">
         <v>130</v>
       </c>
@@ -2997,32 +3957,48 @@
       <c r="F174" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="175" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G174" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="H174" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="I174" s="10"/>
+    </row>
+    <row r="175" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
       <c r="E175" s="3"/>
       <c r="F175" s="3"/>
-    </row>
-    <row r="176" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G175" s="13"/>
+      <c r="H175" s="13"/>
+      <c r="I175" s="11"/>
+    </row>
+    <row r="176" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
       <c r="D176" s="3"/>
       <c r="E176" s="3"/>
       <c r="F176" s="3"/>
-    </row>
-    <row r="177" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G176" s="13"/>
+      <c r="H176" s="13"/>
+      <c r="I176" s="11"/>
+    </row>
+    <row r="177" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="4"/>
       <c r="B177" s="4"/>
       <c r="C177" s="4"/>
       <c r="D177" s="4"/>
       <c r="E177" s="4"/>
       <c r="F177" s="4"/>
-    </row>
-    <row r="178" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G177" s="14"/>
+      <c r="H177" s="14"/>
+      <c r="I177" s="11"/>
+    </row>
+    <row r="178" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="5" t="s">
         <v>135</v>
       </c>
@@ -3041,32 +4017,48 @@
       <c r="F178" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="179" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G178" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="H178" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="I178" s="10"/>
+    </row>
+    <row r="179" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
       <c r="D179" s="3"/>
       <c r="E179" s="3"/>
       <c r="F179" s="3"/>
-    </row>
-    <row r="180" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G179" s="13"/>
+      <c r="H179" s="13"/>
+      <c r="I179" s="11"/>
+    </row>
+    <row r="180" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
       <c r="D180" s="3"/>
       <c r="E180" s="3"/>
       <c r="F180" s="3"/>
-    </row>
-    <row r="181" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G180" s="13"/>
+      <c r="H180" s="13"/>
+      <c r="I180" s="11"/>
+    </row>
+    <row r="181" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="4"/>
       <c r="B181" s="4"/>
       <c r="C181" s="4"/>
       <c r="D181" s="4"/>
       <c r="E181" s="4"/>
       <c r="F181" s="4"/>
-    </row>
-    <row r="182" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G181" s="14"/>
+      <c r="H181" s="14"/>
+      <c r="I181" s="11"/>
+    </row>
+    <row r="182" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="5" t="s">
         <v>138</v>
       </c>
@@ -3085,32 +4077,48 @@
       <c r="F182" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="183" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G182" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="H182" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="I182" s="10"/>
+    </row>
+    <row r="183" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
       <c r="D183" s="3"/>
       <c r="E183" s="3"/>
       <c r="F183" s="3"/>
-    </row>
-    <row r="184" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G183" s="13"/>
+      <c r="H183" s="13"/>
+      <c r="I183" s="11"/>
+    </row>
+    <row r="184" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
       <c r="D184" s="3"/>
       <c r="E184" s="3"/>
       <c r="F184" s="3"/>
-    </row>
-    <row r="185" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G184" s="13"/>
+      <c r="H184" s="13"/>
+      <c r="I184" s="11"/>
+    </row>
+    <row r="185" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="4"/>
       <c r="B185" s="4"/>
       <c r="C185" s="4"/>
       <c r="D185" s="4"/>
       <c r="E185" s="4"/>
       <c r="F185" s="4"/>
-    </row>
-    <row r="186" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G185" s="14"/>
+      <c r="H185" s="14"/>
+      <c r="I185" s="11"/>
+    </row>
+    <row r="186" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="5" t="s">
         <v>141</v>
       </c>
@@ -3129,32 +4137,48 @@
       <c r="F186" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="187" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G186" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="H186" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="I186" s="10"/>
+    </row>
+    <row r="187" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
       <c r="D187" s="3"/>
       <c r="E187" s="3"/>
       <c r="F187" s="3"/>
-    </row>
-    <row r="188" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G187" s="13"/>
+      <c r="H187" s="13"/>
+      <c r="I187" s="11"/>
+    </row>
+    <row r="188" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
       <c r="D188" s="3"/>
       <c r="E188" s="3"/>
       <c r="F188" s="3"/>
-    </row>
-    <row r="189" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G188" s="13"/>
+      <c r="H188" s="13"/>
+      <c r="I188" s="11"/>
+    </row>
+    <row r="189" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="4"/>
       <c r="B189" s="4"/>
       <c r="C189" s="4"/>
       <c r="D189" s="4"/>
       <c r="E189" s="4"/>
       <c r="F189" s="4"/>
-    </row>
-    <row r="190" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G189" s="14"/>
+      <c r="H189" s="14"/>
+      <c r="I189" s="11"/>
+    </row>
+    <row r="190" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="5" t="s">
         <v>142</v>
       </c>
@@ -3173,32 +4197,48 @@
       <c r="F190" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="191" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G190" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="H190" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="I190" s="10"/>
+    </row>
+    <row r="191" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
       <c r="D191" s="3"/>
       <c r="E191" s="3"/>
       <c r="F191" s="3"/>
-    </row>
-    <row r="192" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G191" s="13"/>
+      <c r="H191" s="13"/>
+      <c r="I191" s="11"/>
+    </row>
+    <row r="192" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
       <c r="D192" s="3"/>
       <c r="E192" s="3"/>
       <c r="F192" s="3"/>
-    </row>
-    <row r="193" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G192" s="13"/>
+      <c r="H192" s="13"/>
+      <c r="I192" s="11"/>
+    </row>
+    <row r="193" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="4"/>
       <c r="B193" s="4"/>
       <c r="C193" s="4"/>
       <c r="D193" s="4"/>
       <c r="E193" s="4"/>
       <c r="F193" s="4"/>
-    </row>
-    <row r="194" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G193" s="14"/>
+      <c r="H193" s="14"/>
+      <c r="I193" s="11"/>
+    </row>
+    <row r="194" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="5" t="s">
         <v>145</v>
       </c>
@@ -3217,32 +4257,48 @@
       <c r="F194" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="195" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G194" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H194" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="I194" s="10"/>
+    </row>
+    <row r="195" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
       <c r="D195" s="3"/>
       <c r="E195" s="3"/>
       <c r="F195" s="3"/>
-    </row>
-    <row r="196" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G195" s="13"/>
+      <c r="H195" s="13"/>
+      <c r="I195" s="11"/>
+    </row>
+    <row r="196" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
       <c r="D196" s="3"/>
       <c r="E196" s="3"/>
       <c r="F196" s="3"/>
-    </row>
-    <row r="197" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G196" s="13"/>
+      <c r="H196" s="13"/>
+      <c r="I196" s="11"/>
+    </row>
+    <row r="197" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="4"/>
       <c r="B197" s="4"/>
       <c r="C197" s="4"/>
       <c r="D197" s="4"/>
       <c r="E197" s="4"/>
       <c r="F197" s="4"/>
-    </row>
-    <row r="198" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G197" s="14"/>
+      <c r="H197" s="14"/>
+      <c r="I197" s="11"/>
+    </row>
+    <row r="198" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="5" t="s">
         <v>150</v>
       </c>
@@ -3261,33 +4317,149 @@
       <c r="F198" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="199" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G198" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="H198" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="I198" s="10"/>
+    </row>
+    <row r="199" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
       <c r="E199" s="3"/>
       <c r="F199" s="3"/>
-    </row>
-    <row r="200" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G199" s="13"/>
+      <c r="H199" s="13"/>
+      <c r="I199" s="11"/>
+    </row>
+    <row r="200" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
       <c r="D200" s="3"/>
       <c r="E200" s="3"/>
       <c r="F200" s="3"/>
-    </row>
-    <row r="201" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G200" s="13"/>
+      <c r="H200" s="13"/>
+      <c r="I200" s="11"/>
+    </row>
+    <row r="201" spans="1:9" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="4"/>
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
       <c r="D201" s="4"/>
       <c r="E201" s="4"/>
       <c r="F201" s="4"/>
+      <c r="G201" s="14"/>
+      <c r="H201" s="14"/>
+      <c r="I201" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="300">
+  <mergeCells count="400">
+    <mergeCell ref="G186:G189"/>
+    <mergeCell ref="H186:H189"/>
+    <mergeCell ref="G190:G193"/>
+    <mergeCell ref="H190:H193"/>
+    <mergeCell ref="G194:G197"/>
+    <mergeCell ref="H194:H197"/>
+    <mergeCell ref="G198:G201"/>
+    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="G166:G169"/>
+    <mergeCell ref="H166:H169"/>
+    <mergeCell ref="G170:G173"/>
+    <mergeCell ref="H170:H173"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="H174:H177"/>
+    <mergeCell ref="G178:G181"/>
+    <mergeCell ref="H178:H181"/>
+    <mergeCell ref="G182:G185"/>
+    <mergeCell ref="H182:H185"/>
+    <mergeCell ref="G146:G149"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="G150:G153"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="G154:G157"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="G162:G165"/>
+    <mergeCell ref="H162:H165"/>
+    <mergeCell ref="G126:G129"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="G134:G137"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="G138:G141"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="G142:G145"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="G106:G109"/>
+    <mergeCell ref="H106:H109"/>
+    <mergeCell ref="G110:G113"/>
+    <mergeCell ref="H110:H113"/>
+    <mergeCell ref="G114:G117"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="G118:G121"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="G86:G89"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="G94:G97"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="G98:G101"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="G102:G105"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="G70:G73"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="G74:G77"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="G78:G81"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="G54:G57"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="G62:G65"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="G6:G9"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="G18:G21"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="G30:G33"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="G42:G45"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="G46:G49"/>
     <mergeCell ref="F34:F37"/>
     <mergeCell ref="A34:A37"/>
     <mergeCell ref="B34:B37"/>
@@ -3306,6 +4478,12 @@
     <mergeCell ref="C14:C17"/>
     <mergeCell ref="D14:D17"/>
     <mergeCell ref="E14:E17"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E22:E25"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="C2:C5"/>
@@ -3318,12 +4496,6 @@
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="C6:C9"/>
     <mergeCell ref="D2:D5"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="E22:E25"/>
     <mergeCell ref="F22:F25"/>
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="B18:B21"/>

</xml_diff>